<commit_message>
fix: klik riwayat kunjungan
</commit_message>
<xml_diff>
--- a/FILE EXCEL DISINI/Pasongsongan 25-04-26.xlsx
+++ b/FILE EXCEL DISINI/Pasongsongan 25-04-26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Selenium\FILE EXCEL DISINI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Asisten-Cerdas-Smart-RPA\FILE EXCEL DISINI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6DE640F-0394-4281-B760-A9E0C9230510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FB94C6-9304-46DA-97E0-7FFDF2D5C017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="330" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PASONGSONGAN 25-04-2026" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="113">
   <si>
     <t>PKM PASONGSONGAN</t>
   </si>
@@ -85,9 +85,6 @@
     <t>PASONGSONGAN</t>
   </si>
   <si>
-    <t>TIDAK ADA URINE</t>
-  </si>
-  <si>
     <t>29-04-2026</t>
   </si>
   <si>
@@ -317,6 +314,51 @@
   </si>
   <si>
     <t>STATUS SIMPAN</t>
+  </si>
+  <si>
+    <t>0.9</t>
+  </si>
+  <si>
+    <t>0.7</t>
+  </si>
+  <si>
+    <t>0.6</t>
+  </si>
+  <si>
+    <t>0.8</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>1.4</t>
+  </si>
+  <si>
+    <t>7.6</t>
+  </si>
+  <si>
+    <t>5.0</t>
+  </si>
+  <si>
+    <t>4.7</t>
+  </si>
+  <si>
+    <t>4.8</t>
+  </si>
+  <si>
+    <t>4.4</t>
+  </si>
+  <si>
+    <t>4.9</t>
+  </si>
+  <si>
+    <t>5.3</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>4.6</t>
   </si>
 </sst>
 </file>
@@ -428,7 +470,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -488,9 +530,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -508,6 +547,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -787,40 +832,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T38"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" style="6" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="8" style="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="25.88671875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="8" style="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" style="6" customWidth="1"/>
     <col min="7" max="7" width="14" style="6" customWidth="1"/>
     <col min="8" max="8" width="7" style="6" customWidth="1"/>
-    <col min="9" max="9" width="8.28515625" style="6" customWidth="1"/>
+    <col min="9" max="9" width="8.33203125" style="6" customWidth="1"/>
     <col min="10" max="10" width="7" style="6" customWidth="1"/>
-    <col min="11" max="11" width="7.5703125" style="6" customWidth="1"/>
-    <col min="12" max="12" width="6.7109375" style="6" customWidth="1"/>
-    <col min="13" max="13" width="7.7109375" style="6" customWidth="1"/>
+    <col min="11" max="11" width="7.5546875" style="6" customWidth="1"/>
+    <col min="12" max="12" width="6.6640625" style="6" customWidth="1"/>
+    <col min="13" max="13" width="7.6640625" style="6" customWidth="1"/>
     <col min="14" max="14" width="7" style="6" customWidth="1"/>
-    <col min="15" max="15" width="8.140625" style="6" customWidth="1"/>
-    <col min="16" max="16" width="17.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="41.28515625" style="6" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" style="6" customWidth="1"/>
-    <col min="19" max="19" width="14.140625" style="6" customWidth="1"/>
+    <col min="15" max="15" width="8.109375" style="6" customWidth="1"/>
+    <col min="16" max="16" width="17.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="41.33203125" style="6" customWidth="1"/>
+    <col min="18" max="18" width="16.5546875" style="6" customWidth="1"/>
+    <col min="19" max="19" width="14.109375" style="6" customWidth="1"/>
     <col min="20" max="20" width="33" style="6" customWidth="1"/>
-    <col min="21" max="21" width="14.42578125" style="6" customWidth="1"/>
-    <col min="22" max="16384" width="14.42578125" style="6"/>
+    <col min="21" max="21" width="14.44140625" style="6" customWidth="1"/>
+    <col min="22" max="16384" width="14.44140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="28"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="2"/>
@@ -837,7 +882,7 @@
       <c r="S1" s="5"/>
       <c r="T1" s="5"/>
     </row>
-    <row r="2" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="7">
         <v>46137</v>
@@ -861,7 +906,7 @@
       <c r="S2" s="5"/>
       <c r="T2" s="5"/>
     </row>
-    <row r="3" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>1</v>
       </c>
@@ -911,15 +956,15 @@
         <v>16</v>
       </c>
       <c r="Q3" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="R3" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
     </row>
-    <row r="4" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11">
         <v>1</v>
       </c>
@@ -940,37 +985,49 @@
         <v>18592</v>
       </c>
       <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
+      <c r="I4" s="17">
+        <v>156</v>
+      </c>
+      <c r="J4" s="17">
+        <v>70</v>
+      </c>
+      <c r="K4" s="17">
+        <v>34</v>
+      </c>
+      <c r="L4" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="M4" s="17">
+        <v>54</v>
+      </c>
+      <c r="N4" s="17">
+        <v>88</v>
+      </c>
       <c r="O4" s="17"/>
-      <c r="P4" s="17" t="s">
-        <v>21</v>
+      <c r="P4" s="17">
+        <v>12.1</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R4" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R4" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S4" s="19"/>
       <c r="T4" s="19"/>
     </row>
-    <row r="5" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11">
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" s="11"/>
       <c r="F5" s="15" t="s">
@@ -980,77 +1037,101 @@
         <v>28311</v>
       </c>
       <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
+      <c r="I5" s="17">
+        <v>194</v>
+      </c>
+      <c r="J5" s="17">
+        <v>296</v>
+      </c>
+      <c r="K5" s="17">
+        <v>20</v>
+      </c>
+      <c r="L5" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="M5" s="17">
+        <v>88</v>
+      </c>
+      <c r="N5" s="17">
+        <v>87</v>
+      </c>
       <c r="O5" s="17"/>
       <c r="P5" s="17">
         <v>26.3</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R5" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R5" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S5" s="19"/>
       <c r="T5" s="19"/>
     </row>
-    <row r="6" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11">
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" s="11"/>
       <c r="F6" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G6" s="16">
         <v>28959</v>
       </c>
       <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
+      <c r="I6" s="17">
+        <v>236</v>
+      </c>
+      <c r="J6" s="17">
+        <v>216</v>
+      </c>
+      <c r="K6" s="17">
+        <v>21</v>
+      </c>
+      <c r="L6" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="M6" s="17">
+        <v>59</v>
+      </c>
+      <c r="N6" s="17">
+        <v>134</v>
+      </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17">
         <v>7.4</v>
       </c>
       <c r="Q6" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R6" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R6" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S6" s="19"/>
       <c r="T6" s="19"/>
     </row>
-    <row r="7" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>4</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="15" t="s">
@@ -1060,37 +1141,49 @@
         <v>25247</v>
       </c>
       <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
+      <c r="I7" s="17">
+        <v>182</v>
+      </c>
+      <c r="J7" s="17">
+        <v>163</v>
+      </c>
+      <c r="K7" s="17">
+        <v>17</v>
+      </c>
+      <c r="L7" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M7" s="17">
+        <v>78</v>
+      </c>
+      <c r="N7" s="17">
+        <v>71</v>
+      </c>
       <c r="O7" s="17"/>
-      <c r="P7" s="17" t="s">
-        <v>21</v>
+      <c r="P7" s="17">
+        <v>9.3000000000000007</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R7" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R7" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S7" s="19"/>
       <c r="T7" s="19"/>
     </row>
-    <row r="8" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>5</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="15" t="s">
@@ -1100,37 +1193,49 @@
         <v>21315</v>
       </c>
       <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
+      <c r="I8" s="17">
+        <v>172</v>
+      </c>
+      <c r="J8" s="17">
+        <v>59</v>
+      </c>
+      <c r="K8" s="17">
+        <v>28</v>
+      </c>
+      <c r="L8" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="M8" s="17">
+        <v>67</v>
+      </c>
+      <c r="N8" s="17">
+        <v>93</v>
+      </c>
       <c r="O8" s="17"/>
-      <c r="P8" s="17" t="s">
-        <v>21</v>
+      <c r="P8" s="17">
+        <v>10.199999999999999</v>
       </c>
       <c r="Q8" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R8" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R8" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S8" s="19"/>
       <c r="T8" s="19"/>
     </row>
-    <row r="9" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>6</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="15" t="s">
@@ -1140,77 +1245,101 @@
         <v>30744</v>
       </c>
       <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="18"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
+      <c r="I9" s="17">
+        <v>182</v>
+      </c>
+      <c r="J9" s="17">
+        <v>81</v>
+      </c>
+      <c r="K9" s="17">
+        <v>31</v>
+      </c>
+      <c r="L9" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="M9" s="17">
+        <v>53</v>
+      </c>
+      <c r="N9" s="17">
+        <v>63</v>
+      </c>
       <c r="O9" s="17"/>
-      <c r="P9" s="17" t="s">
-        <v>21</v>
+      <c r="P9" s="17">
+        <v>8.9</v>
       </c>
       <c r="Q9" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R9" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R9" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S9" s="19"/>
       <c r="T9" s="19"/>
     </row>
-    <row r="10" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>7</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E10" s="11"/>
       <c r="F10" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G10" s="16">
         <v>31133</v>
       </c>
       <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
+      <c r="I10" s="17">
+        <v>129</v>
+      </c>
+      <c r="J10" s="17">
+        <v>48</v>
+      </c>
+      <c r="K10" s="17">
+        <v>12</v>
+      </c>
+      <c r="L10" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="M10" s="17">
+        <v>54</v>
+      </c>
+      <c r="N10" s="17">
+        <v>65</v>
+      </c>
       <c r="O10" s="17"/>
-      <c r="P10" s="17" t="s">
-        <v>21</v>
+      <c r="P10" s="17">
+        <v>16.3</v>
       </c>
       <c r="Q10" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R10" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R10" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S10" s="19"/>
       <c r="T10" s="19"/>
     </row>
-    <row r="11" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
         <v>8</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E11" s="11"/>
       <c r="F11" s="15" t="s">
@@ -1220,37 +1349,49 @@
         <v>30860</v>
       </c>
       <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
+      <c r="I11" s="17">
+        <v>271</v>
+      </c>
+      <c r="J11" s="17">
+        <v>384</v>
+      </c>
+      <c r="K11" s="17">
+        <v>16</v>
+      </c>
+      <c r="L11" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M11" s="17">
+        <v>56</v>
+      </c>
+      <c r="N11" s="17">
+        <v>138</v>
+      </c>
       <c r="O11" s="17"/>
       <c r="P11" s="17">
         <v>27.4</v>
       </c>
       <c r="Q11" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R11" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R11" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S11" s="19"/>
       <c r="T11" s="19"/>
     </row>
-    <row r="12" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>9</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E12" s="11"/>
       <c r="F12" s="15" t="s">
@@ -1260,77 +1401,101 @@
         <v>24769</v>
       </c>
       <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
+      <c r="I12" s="17">
+        <v>143</v>
+      </c>
+      <c r="J12" s="17">
+        <v>110</v>
+      </c>
+      <c r="K12" s="17">
+        <v>52</v>
+      </c>
+      <c r="L12" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="M12" s="17">
+        <v>49</v>
+      </c>
+      <c r="N12" s="17">
+        <v>72</v>
+      </c>
       <c r="O12" s="17"/>
       <c r="P12" s="17">
         <v>6.4</v>
       </c>
       <c r="Q12" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R12" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R12" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S12" s="19"/>
       <c r="T12" s="19"/>
     </row>
-    <row r="13" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>10</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G13" s="16">
         <v>20410</v>
       </c>
       <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="18"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="17"/>
+      <c r="I13" s="17">
+        <v>177</v>
+      </c>
+      <c r="J13" s="17">
+        <v>156</v>
+      </c>
+      <c r="K13" s="17">
+        <v>40</v>
+      </c>
+      <c r="L13" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="M13" s="17">
+        <v>67</v>
+      </c>
+      <c r="N13" s="17">
+        <v>79</v>
+      </c>
       <c r="O13" s="17"/>
-      <c r="P13" s="17" t="s">
-        <v>21</v>
+      <c r="P13" s="17">
+        <v>10.199999999999999</v>
       </c>
       <c r="Q13" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R13" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R13" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S13" s="19"/>
       <c r="T13" s="19"/>
     </row>
-    <row r="14" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
         <v>11</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E14" s="11"/>
       <c r="F14" s="15" t="s">
@@ -1340,37 +1505,49 @@
         <v>20271</v>
       </c>
       <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
+      <c r="I14" s="17">
+        <v>140</v>
+      </c>
+      <c r="J14" s="17">
+        <v>68</v>
+      </c>
+      <c r="K14" s="17">
+        <v>22</v>
+      </c>
+      <c r="L14" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="M14" s="17">
+        <v>45</v>
+      </c>
+      <c r="N14" s="17">
+        <v>81</v>
+      </c>
       <c r="O14" s="17"/>
       <c r="P14" s="17">
         <v>5.6</v>
       </c>
       <c r="Q14" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R14" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R14" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S14" s="19"/>
       <c r="T14" s="19"/>
     </row>
-    <row r="15" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
         <v>12</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="15" t="s">
@@ -1380,37 +1557,49 @@
         <v>23193</v>
       </c>
       <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="17"/>
-      <c r="N15" s="17"/>
+      <c r="I15" s="17">
+        <v>184</v>
+      </c>
+      <c r="J15" s="17">
+        <v>186</v>
+      </c>
+      <c r="K15" s="17">
+        <v>28</v>
+      </c>
+      <c r="L15" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="M15" s="17">
+        <v>54</v>
+      </c>
+      <c r="N15" s="17">
+        <v>93</v>
+      </c>
       <c r="O15" s="17"/>
-      <c r="P15" s="17" t="s">
-        <v>21</v>
+      <c r="P15" s="17">
+        <v>13.1</v>
       </c>
       <c r="Q15" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R15" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R15" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S15" s="19"/>
       <c r="T15" s="19"/>
     </row>
-    <row r="16" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
         <v>13</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="15" t="s">
@@ -1420,77 +1609,101 @@
         <v>32848</v>
       </c>
       <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
+      <c r="I16" s="17">
+        <v>242</v>
+      </c>
+      <c r="J16" s="17">
+        <v>555</v>
+      </c>
+      <c r="K16" s="17">
+        <v>31</v>
+      </c>
+      <c r="L16" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M16" s="17">
+        <v>86</v>
+      </c>
+      <c r="N16" s="17">
+        <v>145</v>
+      </c>
       <c r="O16" s="17"/>
-      <c r="P16" s="17" t="s">
-        <v>21</v>
+      <c r="P16" s="17">
+        <v>13.4</v>
       </c>
       <c r="Q16" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R16" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R16" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S16" s="19"/>
       <c r="T16" s="19"/>
     </row>
-    <row r="17" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
         <v>14</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E17" s="11"/>
       <c r="F17" s="15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G17" s="16">
         <v>28348</v>
       </c>
       <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
+      <c r="I17" s="17">
+        <v>249</v>
+      </c>
+      <c r="J17" s="17">
+        <v>76</v>
+      </c>
+      <c r="K17" s="17">
+        <v>21</v>
+      </c>
+      <c r="L17" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M17" s="17">
+        <v>76</v>
+      </c>
+      <c r="N17" s="17">
+        <v>158</v>
+      </c>
       <c r="O17" s="17"/>
-      <c r="P17" s="17" t="s">
-        <v>21</v>
+      <c r="P17" s="17">
+        <v>12.1</v>
       </c>
       <c r="Q17" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R17" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R17" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S17" s="19"/>
       <c r="T17" s="19"/>
     </row>
-    <row r="18" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>15</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E18" s="11"/>
       <c r="F18" s="15" t="s">
@@ -1500,37 +1713,49 @@
         <v>24289</v>
       </c>
       <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
+      <c r="I18" s="17">
+        <v>212</v>
+      </c>
+      <c r="J18" s="17">
+        <v>79</v>
+      </c>
+      <c r="K18" s="17">
+        <v>22</v>
+      </c>
+      <c r="L18" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="M18" s="17">
+        <v>72</v>
+      </c>
+      <c r="N18" s="17">
+        <v>124</v>
+      </c>
       <c r="O18" s="17"/>
-      <c r="P18" s="17" t="s">
-        <v>21</v>
+      <c r="P18" s="17">
+        <v>16.2</v>
       </c>
       <c r="Q18" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R18" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R18" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S18" s="19"/>
       <c r="T18" s="19"/>
     </row>
-    <row r="19" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11">
         <v>16</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E19" s="11"/>
       <c r="F19" s="15" t="s">
@@ -1540,37 +1765,49 @@
         <v>30435</v>
       </c>
       <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
+      <c r="I19" s="17">
+        <v>185</v>
+      </c>
+      <c r="J19" s="17">
+        <v>66</v>
+      </c>
+      <c r="K19" s="17">
+        <v>19</v>
+      </c>
+      <c r="L19" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M19" s="17">
+        <v>84</v>
+      </c>
+      <c r="N19" s="17">
+        <v>88</v>
+      </c>
       <c r="O19" s="17"/>
-      <c r="P19" s="17" t="s">
-        <v>21</v>
+      <c r="P19" s="17">
+        <v>13.3</v>
       </c>
       <c r="Q19" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R19" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R19" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S19" s="19"/>
       <c r="T19" s="19"/>
     </row>
-    <row r="20" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>17</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E20" s="11"/>
       <c r="F20" s="15" t="s">
@@ -1580,37 +1817,49 @@
         <v>25020</v>
       </c>
       <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
+      <c r="I20" s="17">
+        <v>227</v>
+      </c>
+      <c r="J20" s="17">
+        <v>124</v>
+      </c>
+      <c r="K20" s="17">
+        <v>23</v>
+      </c>
+      <c r="L20" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M20" s="17">
+        <v>86</v>
+      </c>
+      <c r="N20" s="17">
+        <v>116</v>
+      </c>
       <c r="O20" s="17"/>
       <c r="P20" s="17">
         <v>6.2</v>
       </c>
       <c r="Q20" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R20" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R20" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S20" s="19"/>
       <c r="T20" s="19"/>
     </row>
-    <row r="21" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>18</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E21" s="11"/>
       <c r="F21" s="15" t="s">
@@ -1620,37 +1869,49 @@
         <v>19980</v>
       </c>
       <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
+      <c r="I21" s="17">
+        <v>187</v>
+      </c>
+      <c r="J21" s="17">
+        <v>166</v>
+      </c>
+      <c r="K21" s="17">
+        <v>19</v>
+      </c>
+      <c r="L21" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="M21" s="17">
+        <v>61</v>
+      </c>
+      <c r="N21" s="17">
+        <v>93</v>
+      </c>
       <c r="O21" s="17"/>
-      <c r="P21" s="17" t="s">
-        <v>21</v>
+      <c r="P21" s="17">
+        <v>12.4</v>
       </c>
       <c r="Q21" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R21" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R21" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S21" s="19"/>
       <c r="T21" s="19"/>
     </row>
-    <row r="22" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>19</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C22" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E22" s="11"/>
       <c r="F22" s="15" t="s">
@@ -1660,37 +1921,49 @@
         <v>18626</v>
       </c>
       <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="17"/>
+      <c r="I22" s="17">
+        <v>225</v>
+      </c>
+      <c r="J22" s="17">
+        <v>258</v>
+      </c>
+      <c r="K22" s="17">
+        <v>20</v>
+      </c>
+      <c r="L22" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M22" s="17">
+        <v>60</v>
+      </c>
+      <c r="N22" s="17">
+        <v>113</v>
+      </c>
       <c r="O22" s="17"/>
-      <c r="P22" s="17" t="s">
-        <v>21</v>
+      <c r="P22" s="17">
+        <v>13.8</v>
       </c>
       <c r="Q22" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R22" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R22" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S22" s="19"/>
       <c r="T22" s="19"/>
     </row>
-    <row r="23" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>20</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E23" s="11"/>
       <c r="F23" s="15" t="s">
@@ -1700,37 +1973,49 @@
         <v>28322</v>
       </c>
       <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
+      <c r="I23" s="17">
+        <v>247</v>
+      </c>
+      <c r="J23" s="17">
+        <v>162</v>
+      </c>
+      <c r="K23" s="17">
+        <v>61</v>
+      </c>
+      <c r="L23" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="M23" s="17">
+        <v>86</v>
+      </c>
+      <c r="N23" s="17">
+        <v>129</v>
+      </c>
       <c r="O23" s="17"/>
       <c r="P23" s="17">
         <v>5.5</v>
       </c>
       <c r="Q23" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R23" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R23" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S23" s="19"/>
       <c r="T23" s="19"/>
     </row>
-    <row r="24" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>21</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E24" s="11"/>
       <c r="F24" s="15" t="s">
@@ -1740,37 +2025,49 @@
         <v>29189</v>
       </c>
       <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="17"/>
-      <c r="N24" s="17"/>
+      <c r="I24" s="17">
+        <v>181</v>
+      </c>
+      <c r="J24" s="17">
+        <v>65</v>
+      </c>
+      <c r="K24" s="17">
+        <v>29</v>
+      </c>
+      <c r="L24" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="M24" s="17">
+        <v>80</v>
+      </c>
+      <c r="N24" s="17">
+        <v>88</v>
+      </c>
       <c r="O24" s="17"/>
-      <c r="P24" s="17" t="s">
-        <v>21</v>
+      <c r="P24" s="17">
+        <v>22.4</v>
       </c>
       <c r="Q24" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R24" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R24" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S24" s="19"/>
       <c r="T24" s="19"/>
     </row>
-    <row r="25" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>22</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E25" s="11"/>
       <c r="F25" s="15" t="s">
@@ -1780,37 +2077,49 @@
         <v>27747</v>
       </c>
       <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="17"/>
-      <c r="N25" s="17"/>
+      <c r="I25" s="17">
+        <v>151</v>
+      </c>
+      <c r="J25" s="17">
+        <v>166</v>
+      </c>
+      <c r="K25" s="17">
+        <v>21</v>
+      </c>
+      <c r="L25" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="M25" s="17">
+        <v>53</v>
+      </c>
+      <c r="N25" s="17">
+        <v>65</v>
+      </c>
       <c r="O25" s="17"/>
-      <c r="P25" s="21">
+      <c r="P25" s="30">
         <v>14.1</v>
       </c>
       <c r="Q25" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R25" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R25" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S25" s="19"/>
       <c r="T25" s="19"/>
     </row>
-    <row r="26" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>23</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E26" s="11"/>
       <c r="F26" s="15" t="s">
@@ -1820,37 +2129,49 @@
         <v>27441</v>
       </c>
       <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="17"/>
-      <c r="N26" s="17"/>
+      <c r="I26" s="17">
+        <v>186</v>
+      </c>
+      <c r="J26" s="17">
+        <v>109</v>
+      </c>
+      <c r="K26" s="17">
+        <v>22</v>
+      </c>
+      <c r="L26" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M26" s="17">
+        <v>83</v>
+      </c>
+      <c r="N26" s="17">
+        <v>81</v>
+      </c>
       <c r="O26" s="17"/>
-      <c r="P26" s="17" t="s">
-        <v>21</v>
+      <c r="P26" s="17">
+        <v>25.3</v>
       </c>
       <c r="Q26" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R26" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R26" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S26" s="19"/>
       <c r="T26" s="19"/>
     </row>
-    <row r="27" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>24</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E27" s="11"/>
       <c r="F27" s="15" t="s">
@@ -1860,37 +2181,49 @@
         <v>26709</v>
       </c>
       <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-      <c r="L27" s="18"/>
-      <c r="M27" s="17"/>
-      <c r="N27" s="17"/>
+      <c r="I27" s="17">
+        <v>317</v>
+      </c>
+      <c r="J27" s="17">
+        <v>267</v>
+      </c>
+      <c r="K27" s="17">
+        <v>17</v>
+      </c>
+      <c r="L27" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="M27" s="17">
+        <v>88</v>
+      </c>
+      <c r="N27" s="17">
+        <v>176</v>
+      </c>
       <c r="O27" s="17"/>
-      <c r="P27" s="17" t="s">
-        <v>21</v>
+      <c r="P27" s="17">
+        <v>16.600000000000001</v>
       </c>
       <c r="Q27" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R27" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R27" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S27" s="19"/>
       <c r="T27" s="19"/>
     </row>
-    <row r="28" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11">
         <v>25</v>
       </c>
       <c r="B28" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="D28" s="14" t="s">
         <v>74</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>75</v>
       </c>
       <c r="E28" s="11"/>
       <c r="F28" s="15" t="s">
@@ -1899,38 +2232,54 @@
       <c r="G28" s="16">
         <v>26307</v>
       </c>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="17"/>
-      <c r="N28" s="17"/>
-      <c r="O28" s="17"/>
-      <c r="P28" s="17" t="s">
-        <v>21</v>
+      <c r="H28" s="17">
+        <v>171</v>
+      </c>
+      <c r="I28" s="17">
+        <v>243</v>
+      </c>
+      <c r="J28" s="17">
+        <v>216</v>
+      </c>
+      <c r="K28" s="17">
+        <v>30</v>
+      </c>
+      <c r="L28" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M28" s="17">
+        <v>84</v>
+      </c>
+      <c r="N28" s="17">
+        <v>116</v>
+      </c>
+      <c r="O28" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="P28" s="17">
+        <v>15.8</v>
       </c>
       <c r="Q28" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R28" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R28" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S28" s="19"/>
       <c r="T28" s="19"/>
     </row>
-    <row r="29" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
         <v>26</v>
       </c>
       <c r="B29" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="14" t="s">
         <v>76</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>77</v>
       </c>
       <c r="E29" s="11"/>
       <c r="F29" s="15" t="s">
@@ -1939,78 +2288,110 @@
       <c r="G29" s="16">
         <v>20669</v>
       </c>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="18"/>
-      <c r="M29" s="17"/>
-      <c r="N29" s="17"/>
-      <c r="O29" s="17"/>
+      <c r="H29" s="17">
+        <v>96</v>
+      </c>
+      <c r="I29" s="17">
+        <v>221</v>
+      </c>
+      <c r="J29" s="17">
+        <v>99</v>
+      </c>
+      <c r="K29" s="17">
+        <v>27</v>
+      </c>
+      <c r="L29" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="M29" s="17">
+        <v>76</v>
+      </c>
+      <c r="N29" s="17">
+        <v>125</v>
+      </c>
+      <c r="O29" s="17" t="s">
+        <v>105</v>
+      </c>
       <c r="P29" s="17">
         <v>7.6</v>
       </c>
       <c r="Q29" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R29" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R29" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S29" s="19"/>
       <c r="T29" s="19"/>
     </row>
-    <row r="30" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11">
         <v>27</v>
       </c>
       <c r="B30" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30" s="14" t="s">
         <v>78</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>79</v>
       </c>
       <c r="E30" s="11"/>
       <c r="F30" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G30" s="16">
         <v>26846</v>
       </c>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="18"/>
-      <c r="M30" s="17"/>
-      <c r="N30" s="17"/>
-      <c r="O30" s="17"/>
-      <c r="P30" s="17" t="s">
-        <v>21</v>
+      <c r="H30" s="17">
+        <v>88</v>
+      </c>
+      <c r="I30" s="17">
+        <v>139</v>
+      </c>
+      <c r="J30" s="17">
+        <v>85</v>
+      </c>
+      <c r="K30" s="17">
+        <v>15</v>
+      </c>
+      <c r="L30" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="M30" s="17">
+        <v>52</v>
+      </c>
+      <c r="N30" s="17">
+        <v>70</v>
+      </c>
+      <c r="O30" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="P30" s="17">
+        <v>17.2</v>
       </c>
       <c r="Q30" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="R30" s="26" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R30" s="25" t="s">
+        <v>22</v>
       </c>
       <c r="S30" s="19"/>
       <c r="T30" s="19"/>
     </row>
-    <row r="31" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="11">
         <v>28</v>
       </c>
       <c r="B31" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D31" s="14" t="s">
         <v>80</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>81</v>
       </c>
       <c r="E31" s="11"/>
       <c r="F31" s="15" t="s">
@@ -2019,36 +2400,52 @@
       <c r="G31" s="16">
         <v>19906</v>
       </c>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="17"/>
-      <c r="P31" s="17" t="s">
-        <v>21</v>
+      <c r="H31" s="31">
+        <v>88</v>
+      </c>
+      <c r="I31" s="17">
+        <v>171</v>
+      </c>
+      <c r="J31" s="17">
+        <v>78</v>
+      </c>
+      <c r="K31" s="17">
+        <v>17</v>
+      </c>
+      <c r="L31" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M31" s="17">
+        <v>74</v>
+      </c>
+      <c r="N31" s="17">
+        <v>81</v>
+      </c>
+      <c r="O31" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="P31" s="17">
+        <v>12.5</v>
       </c>
       <c r="Q31" t="s">
-        <v>22</v>
-      </c>
-      <c r="R31" s="27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="R31" s="26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
         <v>29</v>
       </c>
       <c r="B32" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D32" s="14" t="s">
         <v>82</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>83</v>
       </c>
       <c r="E32" s="11"/>
       <c r="F32" s="15" t="s">
@@ -2057,250 +2454,362 @@
       <c r="G32" s="16">
         <v>36287</v>
       </c>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
-      <c r="K32" s="17"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="17"/>
-      <c r="N32" s="17"/>
-      <c r="O32" s="17"/>
-      <c r="P32" s="17" t="s">
-        <v>21</v>
+      <c r="H32" s="17">
+        <v>91</v>
+      </c>
+      <c r="I32" s="17">
+        <v>135</v>
+      </c>
+      <c r="J32" s="17">
+        <v>101</v>
+      </c>
+      <c r="K32" s="17">
+        <v>19</v>
+      </c>
+      <c r="L32" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M32" s="17">
+        <v>51</v>
+      </c>
+      <c r="N32" s="17">
+        <v>64</v>
+      </c>
+      <c r="O32" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="P32" s="17">
+        <v>8.6999999999999993</v>
       </c>
       <c r="Q32" t="s">
-        <v>22</v>
-      </c>
-      <c r="R32" s="27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="R32" s="26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="11">
         <v>30</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D33" s="14" t="s">
         <v>84</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>85</v>
       </c>
       <c r="E33" s="11"/>
       <c r="F33" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G33" s="16">
         <v>23924</v>
       </c>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="18"/>
-      <c r="M33" s="17"/>
-      <c r="N33" s="17"/>
-      <c r="O33" s="17"/>
-      <c r="P33" s="17" t="s">
-        <v>21</v>
+      <c r="H33" s="17">
+        <v>80</v>
+      </c>
+      <c r="I33" s="17">
+        <v>186</v>
+      </c>
+      <c r="J33" s="17">
+        <v>60</v>
+      </c>
+      <c r="K33" s="17">
+        <v>20</v>
+      </c>
+      <c r="L33" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="M33" s="17">
+        <v>69</v>
+      </c>
+      <c r="N33" s="17">
+        <v>125</v>
+      </c>
+      <c r="O33" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="P33" s="17">
+        <v>12.3</v>
       </c>
       <c r="Q33" t="s">
-        <v>22</v>
-      </c>
-      <c r="R33" s="27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="R33" s="26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11">
         <v>31</v>
       </c>
-      <c r="B34" s="22" t="s">
+      <c r="B34" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="C34" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D34" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="G34" s="24">
+      <c r="E34" s="21"/>
+      <c r="F34" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="G34" s="23">
         <v>26554</v>
       </c>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="22"/>
-      <c r="K34" s="22"/>
-      <c r="L34" s="22"/>
-      <c r="M34" s="22"/>
-      <c r="N34" s="22"/>
-      <c r="O34" s="22"/>
-      <c r="P34" s="17" t="s">
-        <v>21</v>
+      <c r="H34" s="17">
+        <v>95</v>
+      </c>
+      <c r="I34" s="30">
+        <v>216</v>
+      </c>
+      <c r="J34" s="30">
+        <v>359</v>
+      </c>
+      <c r="K34" s="30">
+        <v>32</v>
+      </c>
+      <c r="L34" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="M34" s="30">
+        <v>69</v>
+      </c>
+      <c r="N34" s="30">
+        <v>125</v>
+      </c>
+      <c r="O34" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="P34" s="17">
+        <v>14.5</v>
       </c>
       <c r="Q34" t="s">
-        <v>22</v>
-      </c>
-      <c r="R34" s="27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="R34" s="26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="11">
         <v>32</v>
       </c>
-      <c r="B35" s="22" t="s">
+      <c r="B35" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D35" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="C35" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D35" s="23" t="s">
+      <c r="E35" s="21"/>
+      <c r="F35" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="G35" s="24">
+      <c r="G35" s="23">
         <v>25390</v>
       </c>
-      <c r="H35" s="22"/>
-      <c r="I35" s="22"/>
-      <c r="J35" s="22"/>
-      <c r="K35" s="22"/>
-      <c r="L35" s="22"/>
-      <c r="M35" s="22"/>
-      <c r="N35" s="22"/>
-      <c r="O35" s="22"/>
-      <c r="P35" s="17" t="s">
-        <v>21</v>
+      <c r="H35" s="30">
+        <v>104</v>
+      </c>
+      <c r="I35" s="30">
+        <v>258</v>
+      </c>
+      <c r="J35" s="30">
+        <v>397</v>
+      </c>
+      <c r="K35" s="30">
+        <v>18</v>
+      </c>
+      <c r="L35" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="M35" s="30">
+        <v>62</v>
+      </c>
+      <c r="N35" s="30">
+        <v>117</v>
+      </c>
+      <c r="O35" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="P35" s="17">
+        <v>16.3</v>
       </c>
       <c r="Q35" t="s">
-        <v>22</v>
-      </c>
-      <c r="R35" s="27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="R35" s="26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="11">
         <v>33</v>
       </c>
-      <c r="B36" s="22" t="s">
+      <c r="B36" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D36" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="C36" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D36" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="G36" s="24">
+      <c r="E36" s="21"/>
+      <c r="F36" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="G36" s="23">
         <v>20318</v>
       </c>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22"/>
-      <c r="K36" s="22"/>
-      <c r="L36" s="22"/>
-      <c r="M36" s="22"/>
-      <c r="N36" s="22"/>
-      <c r="O36" s="22"/>
-      <c r="P36" s="17" t="s">
-        <v>21</v>
+      <c r="H36" s="30">
+        <v>90</v>
+      </c>
+      <c r="I36" s="30">
+        <v>242</v>
+      </c>
+      <c r="J36" s="30">
+        <v>111</v>
+      </c>
+      <c r="K36" s="30">
+        <v>32</v>
+      </c>
+      <c r="L36" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="M36" s="30">
+        <v>81</v>
+      </c>
+      <c r="N36" s="30">
+        <v>139</v>
+      </c>
+      <c r="O36" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="P36" s="17">
+        <v>15.2</v>
       </c>
       <c r="Q36" t="s">
-        <v>22</v>
-      </c>
-      <c r="R36" s="27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="37" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="R36" s="26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="11">
         <v>34</v>
       </c>
-      <c r="B37" s="22" t="s">
+      <c r="B37" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="C37" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D37" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="G37" s="24">
+      <c r="E37" s="21"/>
+      <c r="F37" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="G37" s="23">
         <v>29424</v>
       </c>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
-      <c r="J37" s="22"/>
-      <c r="K37" s="22"/>
-      <c r="L37" s="22"/>
-      <c r="M37" s="22"/>
-      <c r="N37" s="22"/>
-      <c r="O37" s="22"/>
-      <c r="P37" s="17" t="s">
-        <v>21</v>
+      <c r="H37" s="30">
+        <v>84</v>
+      </c>
+      <c r="I37" s="30">
+        <v>192</v>
+      </c>
+      <c r="J37" s="30">
+        <v>80</v>
+      </c>
+      <c r="K37" s="30">
+        <v>24</v>
+      </c>
+      <c r="L37" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="M37" s="30">
+        <v>64</v>
+      </c>
+      <c r="N37" s="30">
+        <v>112</v>
+      </c>
+      <c r="O37" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="P37" s="17">
+        <v>18.100000000000001</v>
       </c>
       <c r="Q37" t="s">
-        <v>22</v>
-      </c>
-      <c r="R37" s="27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="38" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="R37" s="26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="11">
         <v>35</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D38" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="C38" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D38" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="G38" s="24">
+      <c r="E38" s="21"/>
+      <c r="F38" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G38" s="23">
         <v>26627</v>
       </c>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
-      <c r="J38" s="22"/>
-      <c r="K38" s="22"/>
-      <c r="L38" s="22"/>
-      <c r="M38" s="22"/>
-      <c r="N38" s="22"/>
-      <c r="O38" s="22"/>
-      <c r="P38" s="21">
+      <c r="H38" s="30">
+        <v>85</v>
+      </c>
+      <c r="I38" s="30">
+        <v>263</v>
+      </c>
+      <c r="J38" s="30">
+        <v>475</v>
+      </c>
+      <c r="K38" s="30">
+        <v>47</v>
+      </c>
+      <c r="L38" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="M38" s="30">
+        <v>66</v>
+      </c>
+      <c r="N38" s="30">
+        <v>102</v>
+      </c>
+      <c r="O38" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="P38" s="30">
         <v>13.7</v>
       </c>
       <c r="Q38" t="s">
-        <v>22</v>
-      </c>
-      <c r="R38" s="27" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="R38" s="26" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>